<commit_message>
Update 26/09/2026 and 27/09/2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="118">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -386,6 +386,12 @@
   </si>
   <si>
     <t xml:space="preserve">Working on my Minor Project </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same working on minor project #1 </t>
+  </si>
+  <si>
+    <t>Uploaded my Minor Project #1</t>
   </si>
 </sst>
 </file>
@@ -3281,49 +3287,97 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+    <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B52" s="14">
+        <v>450</v>
+      </c>
+      <c r="C52" s="14">
+        <v>30</v>
+      </c>
+      <c r="D52" s="14">
+        <v>0</v>
+      </c>
+      <c r="E52" s="14">
+        <v>180</v>
+      </c>
+      <c r="F52" s="14">
+        <v>0</v>
+      </c>
+      <c r="G52" s="14">
+        <v>0</v>
+      </c>
+      <c r="H52" s="14">
+        <v>60</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B53" s="14">
+        <v>540</v>
+      </c>
+      <c r="C53" s="14">
+        <v>30</v>
+      </c>
+      <c r="D53" s="14">
+        <v>0</v>
+      </c>
+      <c r="E53" s="14">
+        <v>60</v>
+      </c>
+      <c r="F53" s="14">
+        <v>0</v>
+      </c>
+      <c r="G53" s="14">
+        <v>0</v>
+      </c>
+      <c r="H53" s="14">
+        <v>120</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
+        <v>690</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N53" s="17" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="13"/>

</xml_diff>

<commit_message>
Update for 28, 29 and 30 September 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="119">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -392,6 +392,9 @@
   </si>
   <si>
     <t>Uploaded my Minor Project #1</t>
+  </si>
+  <si>
+    <t>preparation for mid term exam</t>
   </si>
 </sst>
 </file>
@@ -3379,71 +3382,143 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+    <row r="54" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B54" s="14">
+        <v>500</v>
+      </c>
+      <c r="C54" s="14">
+        <v>60</v>
+      </c>
+      <c r="D54" s="14">
+        <v>240</v>
+      </c>
+      <c r="E54" s="14">
+        <v>60</v>
+      </c>
+      <c r="F54" s="14">
+        <v>0</v>
+      </c>
+      <c r="G54" s="14">
+        <v>0</v>
+      </c>
+      <c r="H54" s="14">
+        <v>30</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="17"/>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+        <v>550</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N54" s="17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B55" s="14">
+        <v>500</v>
+      </c>
+      <c r="C55" s="14">
+        <v>60</v>
+      </c>
+      <c r="D55" s="14">
+        <v>240</v>
+      </c>
+      <c r="E55" s="14">
+        <v>60</v>
+      </c>
+      <c r="F55" s="14">
+        <v>0</v>
+      </c>
+      <c r="G55" s="14">
+        <v>0</v>
+      </c>
+      <c r="H55" s="14">
+        <v>30</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="17"/>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="13"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
+        <v>550</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M55" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N55" s="17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="13">
+        <v>46295</v>
+      </c>
+      <c r="B56" s="14">
+        <v>500</v>
+      </c>
+      <c r="C56" s="14">
+        <v>60</v>
+      </c>
+      <c r="D56" s="14">
+        <v>240</v>
+      </c>
+      <c r="E56" s="14">
+        <v>60</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14">
+        <v>30</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-      <c r="N56" s="17"/>
+        <v>550</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N56" s="17" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="13"/>

</xml_diff>

<commit_message>
Update of 1st october and 2nd October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="123">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -303,9 +303,6 @@
     <t>Today I run so fast in track, and after coming back I have done some logic building questions to code more better and revise today's topic of Database and Communication</t>
   </si>
   <si>
-    <t>September</t>
-  </si>
-  <si>
     <t>Preparing for Data Networking and Communicationn CA exam, and other personal works also</t>
   </si>
   <si>
@@ -395,6 +392,21 @@
   </si>
   <si>
     <t>preparation for mid term exam</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>Fever and today I clean by shoes, iron some formal shirts and pants</t>
+  </si>
+  <si>
+    <t>Holiday(College leave)</t>
+  </si>
+  <si>
+    <t>Same fever and done some little bit study for my Mid term</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1064,7 @@
     <col min="2" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
@@ -1109,7 +1121,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G3" s="21"/>
     </row>
@@ -2183,7 +2195,7 @@
         <v>69</v>
       </c>
       <c r="N27" s="17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="195" x14ac:dyDescent="0.25">
@@ -2229,7 +2241,7 @@
         <v>51</v>
       </c>
       <c r="N28" s="17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2275,7 +2287,7 @@
         <v>51</v>
       </c>
       <c r="N29" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2321,7 +2333,7 @@
         <v>51</v>
       </c>
       <c r="N30" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="75" x14ac:dyDescent="0.25">
@@ -2367,7 +2379,7 @@
         <v>69</v>
       </c>
       <c r="N31" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2413,7 +2425,7 @@
         <v>51</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2459,7 +2471,7 @@
         <v>51</v>
       </c>
       <c r="N33" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2505,7 +2517,7 @@
         <v>58</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -2551,7 +2563,7 @@
         <v>51</v>
       </c>
       <c r="N35" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2597,7 +2609,7 @@
         <v>58</v>
       </c>
       <c r="N36" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2643,7 +2655,7 @@
         <v>51</v>
       </c>
       <c r="N37" s="17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="171" customHeight="1" x14ac:dyDescent="0.25">
@@ -2666,7 +2678,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H38" s="14">
         <v>510</v>
@@ -2689,7 +2701,7 @@
         <v>58</v>
       </c>
       <c r="N38" s="17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="300" x14ac:dyDescent="0.25">
@@ -2735,7 +2747,7 @@
         <v>58</v>
       </c>
       <c r="N39" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -2781,7 +2793,7 @@
         <v>51</v>
       </c>
       <c r="N40" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="75" x14ac:dyDescent="0.25">
@@ -2827,7 +2839,7 @@
         <v>51</v>
       </c>
       <c r="N41" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -2873,7 +2885,7 @@
         <v>51</v>
       </c>
       <c r="N42" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2919,7 +2931,7 @@
         <v>58</v>
       </c>
       <c r="N43" s="17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2965,7 +2977,7 @@
         <v>51</v>
       </c>
       <c r="N44" s="17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2988,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H45" s="14">
         <v>180</v>
@@ -3011,7 +3023,7 @@
         <v>58</v>
       </c>
       <c r="N45" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -3057,7 +3069,7 @@
         <v>51</v>
       </c>
       <c r="N46" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -3103,7 +3115,7 @@
         <v>51</v>
       </c>
       <c r="N47" s="17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="105" x14ac:dyDescent="0.25">
@@ -3149,7 +3161,7 @@
         <v>58</v>
       </c>
       <c r="N48" s="17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -3195,7 +3207,7 @@
         <v>51</v>
       </c>
       <c r="N49" s="17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -3241,7 +3253,7 @@
         <v>58</v>
       </c>
       <c r="N50" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -3287,7 +3299,7 @@
         <v>58</v>
       </c>
       <c r="N51" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -3333,7 +3345,7 @@
         <v>51</v>
       </c>
       <c r="N52" s="17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -3355,8 +3367,8 @@
       <c r="F53" s="14">
         <v>0</v>
       </c>
-      <c r="G53" s="14">
-        <v>0</v>
+      <c r="G53" s="14" t="s">
+        <v>121</v>
       </c>
       <c r="H53" s="14">
         <v>120</v>
@@ -3379,7 +3391,7 @@
         <v>58</v>
       </c>
       <c r="N53" s="17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -3401,8 +3413,8 @@
       <c r="F54" s="14">
         <v>0</v>
       </c>
-      <c r="G54" s="14">
-        <v>0</v>
+      <c r="G54" s="14" t="s">
+        <v>121</v>
       </c>
       <c r="H54" s="14">
         <v>30</v>
@@ -3425,7 +3437,7 @@
         <v>51</v>
       </c>
       <c r="N54" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -3447,8 +3459,8 @@
       <c r="F55" s="14">
         <v>0</v>
       </c>
-      <c r="G55" s="14">
-        <v>0</v>
+      <c r="G55" s="14" t="s">
+        <v>121</v>
       </c>
       <c r="H55" s="14">
         <v>30</v>
@@ -3471,7 +3483,7 @@
         <v>58</v>
       </c>
       <c r="N55" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -3493,8 +3505,8 @@
       <c r="F56" s="14">
         <v>0</v>
       </c>
-      <c r="G56" s="14">
-        <v>0</v>
+      <c r="G56" s="14" t="s">
+        <v>121</v>
       </c>
       <c r="H56" s="14">
         <v>30</v>
@@ -3517,52 +3529,100 @@
         <v>51</v>
       </c>
       <c r="N56" s="17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A57" s="13"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="15" t="str">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A57" s="13">
+        <v>46296</v>
+      </c>
+      <c r="B57" s="14">
+        <v>450</v>
+      </c>
+      <c r="C57" s="14">
+        <v>30</v>
+      </c>
+      <c r="D57" s="14">
+        <v>0</v>
+      </c>
+      <c r="E57" s="14">
+        <v>0</v>
+      </c>
+      <c r="F57" s="14">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H57" s="14">
+        <v>30</v>
+      </c>
+      <c r="I57" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
+        <v>510</v>
+      </c>
+      <c r="J57" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
-      <c r="N57" s="17"/>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A58" s="13"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="15" t="str">
+        <v>930</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="M57" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N57" s="17" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A58" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B58" s="14">
+        <v>450</v>
+      </c>
+      <c r="C58" s="14">
+        <v>30</v>
+      </c>
+      <c r="D58" s="14">
+        <v>60</v>
+      </c>
+      <c r="E58" s="14">
+        <v>60</v>
+      </c>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H58" s="14">
+        <v>0</v>
+      </c>
+      <c r="I58" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J58" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="17"/>
+        <v>840</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N58" s="17" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13"/>

</xml_diff>

<commit_message>
Update of 3rd October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="123">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3624,27 +3624,51 @@
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="13"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="15" t="str">
+    <row r="59" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A59" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B59" s="14">
+        <v>450</v>
+      </c>
+      <c r="C59" s="14">
+        <v>30</v>
+      </c>
+      <c r="D59" s="14">
+        <v>60</v>
+      </c>
+      <c r="E59" s="14">
+        <v>60</v>
+      </c>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H59" s="14">
+        <v>0</v>
+      </c>
+      <c r="I59" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J59" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-      <c r="N59" s="17"/>
+        <v>840</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N59" s="17" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="13"/>

</xml_diff>

<commit_message>
Update 4th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="124">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -407,6 +407,9 @@
   </si>
   <si>
     <t>Same fever and done some little bit study for my Mid term</t>
+  </si>
+  <si>
+    <t>Feeling better than yesterday, And preparing for Mid term Exam</t>
   </si>
 </sst>
 </file>
@@ -3670,27 +3673,51 @@
         <v>122</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A60" s="13"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="14"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="15" t="str">
+    <row r="60" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A60" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B60" s="14">
+        <v>550</v>
+      </c>
+      <c r="C60" s="14">
+        <v>30</v>
+      </c>
+      <c r="D60" s="14">
+        <v>60</v>
+      </c>
+      <c r="E60" s="14">
+        <v>60</v>
+      </c>
+      <c r="F60" s="14">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H60" s="14">
+        <v>60</v>
+      </c>
+      <c r="I60" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="15" t="str">
+        <v>760</v>
+      </c>
+      <c r="J60" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="17"/>
+        <v>680</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N60" s="17" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13"/>

</xml_diff>

<commit_message>
Update of 5th and 6th of October
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="127">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -410,6 +410,15 @@
   </si>
   <si>
     <t>Feeling better than yesterday, And preparing for Mid term Exam</t>
+  </si>
+  <si>
+    <t>Online Class (4)</t>
+  </si>
+  <si>
+    <t>Preparing for MTE</t>
+  </si>
+  <si>
+    <t>Online Class (5)</t>
   </si>
 </sst>
 </file>
@@ -3720,48 +3729,96 @@
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A61" s="13"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="15" t="str">
+      <c r="A61" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B61" s="14">
+        <v>450</v>
+      </c>
+      <c r="C61" s="14">
+        <v>30</v>
+      </c>
+      <c r="D61" s="14">
+        <v>30</v>
+      </c>
+      <c r="E61" s="14">
+        <v>60</v>
+      </c>
+      <c r="F61" s="14">
+        <v>200</v>
+      </c>
+      <c r="G61" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="H61" s="14">
+        <v>60</v>
+      </c>
+      <c r="I61" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J61" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="17"/>
+        <v>610</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L61" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N61" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A62" s="13"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="15" t="str">
+      <c r="A62" s="13">
+        <v>46301</v>
+      </c>
+      <c r="B62" s="14">
+        <v>450</v>
+      </c>
+      <c r="C62" s="14">
+        <v>30</v>
+      </c>
+      <c r="D62" s="14">
+        <v>60</v>
+      </c>
+      <c r="E62" s="14">
+        <v>60</v>
+      </c>
+      <c r="F62" s="14">
+        <v>250</v>
+      </c>
+      <c r="G62" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H62" s="14">
+        <v>60</v>
+      </c>
+      <c r="I62" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J62" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="17"/>
+        <v>530</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L62" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N62" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="13"/>

</xml_diff>

<commit_message>
Updte 7th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="127">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3821,26 +3821,50 @@
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A63" s="13"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="15" t="str">
+      <c r="A63" s="13">
+        <v>46302</v>
+      </c>
+      <c r="B63" s="14">
+        <v>420</v>
+      </c>
+      <c r="C63" s="14">
+        <v>60</v>
+      </c>
+      <c r="D63" s="14">
+        <v>60</v>
+      </c>
+      <c r="E63" s="14">
+        <v>60</v>
+      </c>
+      <c r="F63" s="14">
+        <v>250</v>
+      </c>
+      <c r="G63" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H63" s="14">
+        <v>120</v>
+      </c>
+      <c r="I63" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J63" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
-      <c r="N63" s="17"/>
+        <v>470</v>
+      </c>
+      <c r="K63" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L63" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N63" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="13"/>

</xml_diff>

<commit_message>
UPdate of 8th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="128">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -419,6 +419,9 @@
   </si>
   <si>
     <t>Online Class (5)</t>
+  </si>
+  <si>
+    <t>College Leave</t>
   </si>
 </sst>
 </file>
@@ -3867,26 +3870,50 @@
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A64" s="13"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="15" t="str">
+      <c r="A64" s="13">
+        <v>46303</v>
+      </c>
+      <c r="B64" s="14">
+        <v>420</v>
+      </c>
+      <c r="C64" s="14">
+        <v>60</v>
+      </c>
+      <c r="D64" s="14">
+        <v>60</v>
+      </c>
+      <c r="E64" s="14">
+        <v>60</v>
+      </c>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H64" s="14">
+        <v>120</v>
+      </c>
+      <c r="I64" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J64" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-      <c r="N64" s="17"/>
+        <v>720</v>
+      </c>
+      <c r="K64" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L64" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N64" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="13"/>

</xml_diff>

<commit_message>
Update 9th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\776\CAP776-Daily-Work\Introudction in Pyhton EXCEL\Introudction in Pyhton EXCEL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\776\CAP776-Daily-Work\Introudction in Pyhton EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="128">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3916,26 +3916,50 @@
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A65" s="13"/>
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
-      <c r="H65" s="14"/>
-      <c r="I65" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-      <c r="N65" s="17"/>
+      <c r="A65" s="13">
+        <v>46304</v>
+      </c>
+      <c r="B65" s="14">
+        <v>420</v>
+      </c>
+      <c r="C65" s="14">
+        <v>60</v>
+      </c>
+      <c r="D65" s="14">
+        <v>60</v>
+      </c>
+      <c r="E65" s="14">
+        <v>0</v>
+      </c>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H65" s="14">
+        <v>121</v>
+      </c>
+      <c r="I65" s="15">
+        <f t="shared" ref="I65" si="2">IF(SUM(B65:F65,H65)=0,"",SUM(B65:F65,H65))</f>
+        <v>661</v>
+      </c>
+      <c r="J65" s="15">
+        <f t="shared" ref="J65" si="3">IF(I65="","",1440-I65)</f>
+        <v>779</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L65" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N65" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="13"/>
@@ -4035,11 +4059,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="2">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="4">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="3">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="5">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -4057,11 +4081,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4079,11 +4103,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4101,11 +4125,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4123,11 +4147,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4145,11 +4169,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4167,11 +4191,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4189,11 +4213,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4211,11 +4235,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4233,11 +4257,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4255,11 +4279,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4277,11 +4301,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4299,11 +4323,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4321,11 +4345,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4343,11 +4367,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4365,11 +4389,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4387,11 +4411,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4409,11 +4433,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4431,11 +4455,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4453,11 +4477,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4475,11 +4499,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4497,11 +4521,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4519,11 +4543,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4541,11 +4565,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4563,11 +4587,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4585,11 +4609,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4607,11 +4631,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4629,11 +4653,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4651,11 +4675,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4673,11 +4697,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4695,11 +4719,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4717,11 +4741,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4739,11 +4763,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4761,11 +4785,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4783,11 +4807,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4805,11 +4829,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4827,11 +4851,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4849,11 +4873,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4871,11 +4895,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4893,11 +4917,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4915,11 +4939,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4937,11 +4961,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4959,11 +4983,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -4981,11 +5005,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5003,11 +5027,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5025,11 +5049,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5047,11 +5071,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5069,11 +5093,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5091,11 +5115,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5113,11 +5137,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5135,11 +5159,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5157,11 +5181,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5179,11 +5203,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5201,11 +5225,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5223,11 +5247,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5245,11 +5269,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5267,11 +5291,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5289,11 +5313,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5311,11 +5335,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5333,11 +5357,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5355,11 +5379,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5377,11 +5401,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5399,11 +5423,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5421,11 +5445,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5443,11 +5467,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="4">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="6">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="5">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="7">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5465,11 +5489,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5487,11 +5511,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5509,11 +5533,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5531,11 +5555,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5553,11 +5577,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5575,11 +5599,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5597,11 +5621,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5619,11 +5643,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5641,11 +5665,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5663,11 +5687,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5685,11 +5709,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5707,11 +5731,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5729,11 +5753,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5751,11 +5775,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5773,11 +5797,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5795,11 +5819,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5817,11 +5841,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5839,11 +5863,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5861,11 +5885,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5883,11 +5907,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5905,11 +5929,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5927,11 +5951,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5949,11 +5973,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5971,11 +5995,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -5993,11 +6017,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6015,11 +6039,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6037,11 +6061,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6059,11 +6083,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6081,11 +6105,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6103,11 +6127,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6125,11 +6149,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6147,11 +6171,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6169,11 +6193,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6191,11 +6215,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6213,11 +6237,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6235,11 +6259,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6257,11 +6281,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6279,11 +6303,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6301,11 +6325,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6323,11 +6347,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6345,11 +6369,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6367,11 +6391,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6389,11 +6413,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6411,11 +6435,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6433,11 +6457,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6455,11 +6479,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6477,11 +6501,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6499,11 +6523,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6521,11 +6545,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6543,11 +6567,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6565,11 +6589,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6587,11 +6611,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6609,11 +6633,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6631,11 +6655,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6653,11 +6677,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6675,11 +6699,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6697,11 +6721,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6719,11 +6743,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6741,11 +6765,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6763,11 +6787,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6785,11 +6809,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6807,11 +6831,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6829,11 +6853,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6851,11 +6875,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="6">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="8">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="7">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="9">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6873,11 +6897,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6895,11 +6919,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6917,11 +6941,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6939,11 +6963,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6961,11 +6985,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -6983,11 +7007,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7005,11 +7029,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7027,11 +7051,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7049,11 +7073,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7071,11 +7095,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7093,11 +7117,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7115,11 +7139,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7137,11 +7161,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7159,11 +7183,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7181,11 +7205,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7203,11 +7227,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7225,11 +7249,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7247,11 +7271,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7269,11 +7293,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7291,11 +7315,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7313,11 +7337,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7335,11 +7359,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7357,11 +7381,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7379,11 +7403,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7401,11 +7425,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7423,11 +7447,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7445,11 +7469,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7467,11 +7491,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7489,11 +7513,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7511,11 +7535,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7533,11 +7557,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7555,11 +7579,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7577,11 +7601,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7599,11 +7623,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7621,11 +7645,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7643,11 +7667,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7665,11 +7689,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7687,11 +7711,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7709,11 +7733,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7731,11 +7755,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7753,11 +7777,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7775,11 +7799,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7797,11 +7821,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7819,11 +7843,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7841,11 +7865,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7863,11 +7887,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7885,11 +7909,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7907,11 +7931,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7929,11 +7953,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7951,11 +7975,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7973,11 +7997,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -7995,11 +8019,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8017,11 +8041,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8039,11 +8063,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8061,11 +8085,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8083,11 +8107,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8105,11 +8129,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8127,11 +8151,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8149,11 +8173,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8171,11 +8195,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8193,11 +8217,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8215,11 +8239,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8237,11 +8261,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8259,11 +8283,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="8">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="10">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="9">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="11">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8281,11 +8305,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8303,11 +8327,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8325,11 +8349,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8347,11 +8371,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8369,11 +8393,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8391,11 +8415,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8413,11 +8437,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8435,11 +8459,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8457,11 +8481,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8479,11 +8503,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8501,11 +8525,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8523,11 +8547,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8545,11 +8569,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8567,11 +8591,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8589,11 +8613,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8611,11 +8635,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8633,11 +8657,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8655,11 +8679,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8677,11 +8701,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8699,11 +8723,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8721,11 +8745,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8743,11 +8767,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8765,11 +8789,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8787,11 +8811,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8809,11 +8833,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8831,11 +8855,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8853,11 +8877,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8875,11 +8899,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8897,11 +8921,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8919,11 +8943,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8941,11 +8965,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8963,11 +8987,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -8985,11 +9009,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9007,11 +9031,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9029,11 +9053,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9051,11 +9075,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9073,11 +9097,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9095,11 +9119,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9117,11 +9141,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9139,11 +9163,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9161,11 +9185,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9183,11 +9207,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9205,11 +9229,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9227,11 +9251,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9249,11 +9273,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9271,11 +9295,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9293,11 +9317,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9315,11 +9339,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9337,11 +9361,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9359,11 +9383,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9381,11 +9405,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9403,11 +9427,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9425,11 +9449,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9447,11 +9471,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9469,11 +9493,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9491,11 +9515,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9513,11 +9537,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9535,11 +9559,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9557,11 +9581,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9579,11 +9603,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9601,11 +9625,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9623,11 +9647,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9645,11 +9669,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9667,11 +9691,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="10">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="12">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="11">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="13">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9689,11 +9713,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9711,11 +9735,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9733,11 +9757,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9755,11 +9779,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9777,11 +9801,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9799,11 +9823,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9821,11 +9845,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9843,11 +9867,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9865,11 +9889,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9887,11 +9911,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9909,11 +9933,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9931,11 +9955,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9953,11 +9977,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9975,11 +9999,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -9997,11 +10021,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10019,11 +10043,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10041,11 +10065,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10063,11 +10087,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10085,11 +10109,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10107,11 +10131,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10129,11 +10153,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10151,11 +10175,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10173,11 +10197,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10195,11 +10219,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10217,11 +10241,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10239,11 +10263,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10261,11 +10285,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10283,11 +10307,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10305,11 +10329,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10327,11 +10351,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10349,11 +10373,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10371,11 +10395,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10393,11 +10417,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10415,11 +10439,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10437,11 +10461,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10459,11 +10483,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10481,11 +10505,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10503,11 +10527,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10525,11 +10549,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10547,11 +10571,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10569,11 +10593,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10591,11 +10615,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10613,11 +10637,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10635,11 +10659,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10657,11 +10681,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10679,11 +10703,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10701,11 +10725,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10723,11 +10747,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10745,11 +10769,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10767,11 +10791,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10789,11 +10813,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10811,11 +10835,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10833,11 +10857,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10855,11 +10879,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10877,11 +10901,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10899,11 +10923,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10921,11 +10945,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10943,11 +10967,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10965,11 +10989,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -10987,11 +11011,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11009,11 +11033,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11031,11 +11055,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11053,11 +11077,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11075,11 +11099,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="14">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="13">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="15">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11097,11 +11121,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11119,11 +11143,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11141,11 +11165,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11163,11 +11187,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11185,11 +11209,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11207,11 +11231,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11229,11 +11253,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11251,11 +11275,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11273,11 +11297,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11295,11 +11319,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11317,11 +11341,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
Update 10th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="128">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3962,26 +3962,50 @@
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A66" s="13"/>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
-      <c r="G66" s="14"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-      <c r="N66" s="17"/>
+      <c r="A66" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B66" s="14">
+        <v>420</v>
+      </c>
+      <c r="C66" s="14">
+        <v>60</v>
+      </c>
+      <c r="D66" s="14">
+        <v>60</v>
+      </c>
+      <c r="E66" s="14">
+        <v>20</v>
+      </c>
+      <c r="F66" s="14">
+        <v>0</v>
+      </c>
+      <c r="G66" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H66" s="14">
+        <v>122</v>
+      </c>
+      <c r="I66" s="15">
+        <f t="shared" ref="I66" si="4">IF(SUM(B66:F66,H66)=0,"",SUM(B66:F66,H66))</f>
+        <v>682</v>
+      </c>
+      <c r="J66" s="15">
+        <f t="shared" ref="J66" si="5">IF(I66="","",1440-I66)</f>
+        <v>758</v>
+      </c>
+      <c r="K66" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L66" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N66" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="13"/>
@@ -4059,11 +4083,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="4">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" ref="I70:I133" si="6">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="5">IF(I70="","",1440-I70)</f>
+        <f t="shared" ref="J70:J133" si="7">IF(I70="","",1440-I70)</f>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -4081,11 +4105,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4103,11 +4127,11 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J72" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K72" s="16"/>
@@ -4125,11 +4149,11 @@
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
       <c r="I73" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J73" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K73" s="16"/>
@@ -4147,11 +4171,11 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J74" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K74" s="16"/>
@@ -4169,11 +4193,11 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J75" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K75" s="16"/>
@@ -4191,11 +4215,11 @@
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
       <c r="I76" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J76" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K76" s="16"/>
@@ -4213,11 +4237,11 @@
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
       <c r="I77" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J77" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K77" s="16"/>
@@ -4235,11 +4259,11 @@
       <c r="G78" s="14"/>
       <c r="H78" s="14"/>
       <c r="I78" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J78" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K78" s="16"/>
@@ -4257,11 +4281,11 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J79" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K79" s="16"/>
@@ -4279,11 +4303,11 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J80" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K80" s="16"/>
@@ -4301,11 +4325,11 @@
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J81" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K81" s="16"/>
@@ -4323,11 +4347,11 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J82" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K82" s="16"/>
@@ -4345,11 +4369,11 @@
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
       <c r="I83" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J83" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K83" s="16"/>
@@ -4367,11 +4391,11 @@
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
       <c r="I84" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J84" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K84" s="16"/>
@@ -4389,11 +4413,11 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J85" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K85" s="16"/>
@@ -4411,11 +4435,11 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J86" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K86" s="16"/>
@@ -4433,11 +4457,11 @@
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
       <c r="I87" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J87" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K87" s="16"/>
@@ -4455,11 +4479,11 @@
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
       <c r="I88" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J88" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K88" s="16"/>
@@ -4477,11 +4501,11 @@
       <c r="G89" s="14"/>
       <c r="H89" s="14"/>
       <c r="I89" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J89" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K89" s="16"/>
@@ -4499,11 +4523,11 @@
       <c r="G90" s="14"/>
       <c r="H90" s="14"/>
       <c r="I90" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J90" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K90" s="16"/>
@@ -4521,11 +4545,11 @@
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
       <c r="I91" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J91" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K91" s="16"/>
@@ -4543,11 +4567,11 @@
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
       <c r="I92" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J92" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K92" s="16"/>
@@ -4565,11 +4589,11 @@
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J93" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K93" s="16"/>
@@ -4587,11 +4611,11 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J94" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K94" s="16"/>
@@ -4609,11 +4633,11 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J95" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K95" s="16"/>
@@ -4631,11 +4655,11 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J96" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K96" s="16"/>
@@ -4653,11 +4677,11 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J97" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K97" s="16"/>
@@ -4675,11 +4699,11 @@
       <c r="G98" s="14"/>
       <c r="H98" s="14"/>
       <c r="I98" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J98" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K98" s="16"/>
@@ -4697,11 +4721,11 @@
       <c r="G99" s="14"/>
       <c r="H99" s="14"/>
       <c r="I99" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J99" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K99" s="16"/>
@@ -4719,11 +4743,11 @@
       <c r="G100" s="14"/>
       <c r="H100" s="14"/>
       <c r="I100" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J100" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K100" s="16"/>
@@ -4741,11 +4765,11 @@
       <c r="G101" s="14"/>
       <c r="H101" s="14"/>
       <c r="I101" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J101" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K101" s="16"/>
@@ -4763,11 +4787,11 @@
       <c r="G102" s="14"/>
       <c r="H102" s="14"/>
       <c r="I102" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J102" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K102" s="16"/>
@@ -4785,11 +4809,11 @@
       <c r="G103" s="14"/>
       <c r="H103" s="14"/>
       <c r="I103" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J103" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K103" s="16"/>
@@ -4807,11 +4831,11 @@
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
       <c r="I104" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J104" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K104" s="16"/>
@@ -4829,11 +4853,11 @@
       <c r="G105" s="14"/>
       <c r="H105" s="14"/>
       <c r="I105" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J105" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K105" s="16"/>
@@ -4851,11 +4875,11 @@
       <c r="G106" s="14"/>
       <c r="H106" s="14"/>
       <c r="I106" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J106" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K106" s="16"/>
@@ -4873,11 +4897,11 @@
       <c r="G107" s="14"/>
       <c r="H107" s="14"/>
       <c r="I107" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J107" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K107" s="16"/>
@@ -4895,11 +4919,11 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J108" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K108" s="16"/>
@@ -4917,11 +4941,11 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J109" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K109" s="16"/>
@@ -4939,11 +4963,11 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J110" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K110" s="16"/>
@@ -4961,11 +4985,11 @@
       <c r="G111" s="14"/>
       <c r="H111" s="14"/>
       <c r="I111" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J111" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K111" s="16"/>
@@ -4983,11 +5007,11 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J112" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K112" s="16"/>
@@ -5005,11 +5029,11 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J113" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K113" s="16"/>
@@ -5027,11 +5051,11 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J114" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K114" s="16"/>
@@ -5049,11 +5073,11 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J115" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K115" s="16"/>
@@ -5071,11 +5095,11 @@
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
       <c r="I116" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J116" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K116" s="16"/>
@@ -5093,11 +5117,11 @@
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
       <c r="I117" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J117" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K117" s="16"/>
@@ -5115,11 +5139,11 @@
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
       <c r="I118" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J118" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K118" s="16"/>
@@ -5137,11 +5161,11 @@
       <c r="G119" s="14"/>
       <c r="H119" s="14"/>
       <c r="I119" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J119" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K119" s="16"/>
@@ -5159,11 +5183,11 @@
       <c r="G120" s="14"/>
       <c r="H120" s="14"/>
       <c r="I120" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J120" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K120" s="16"/>
@@ -5181,11 +5205,11 @@
       <c r="G121" s="14"/>
       <c r="H121" s="14"/>
       <c r="I121" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J121" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K121" s="16"/>
@@ -5203,11 +5227,11 @@
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
       <c r="I122" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J122" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K122" s="16"/>
@@ -5225,11 +5249,11 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J123" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K123" s="16"/>
@@ -5247,11 +5271,11 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J124" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K124" s="16"/>
@@ -5269,11 +5293,11 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J125" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K125" s="16"/>
@@ -5291,11 +5315,11 @@
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
       <c r="I126" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J126" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K126" s="16"/>
@@ -5313,11 +5337,11 @@
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J127" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K127" s="16"/>
@@ -5335,11 +5359,11 @@
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
       <c r="I128" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J128" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K128" s="16"/>
@@ -5357,11 +5381,11 @@
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
       <c r="I129" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J129" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K129" s="16"/>
@@ -5379,11 +5403,11 @@
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
       <c r="I130" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J130" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K130" s="16"/>
@@ -5401,11 +5425,11 @@
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
       <c r="I131" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J131" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K131" s="16"/>
@@ -5423,11 +5447,11 @@
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
       <c r="I132" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J132" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K132" s="16"/>
@@ -5445,11 +5469,11 @@
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
       <c r="I133" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J133" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K133" s="16"/>
@@ -5467,11 +5491,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="6">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" ref="I134:I197" si="8">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="7">IF(I134="","",1440-I134)</f>
+        <f t="shared" ref="J134:J197" si="9">IF(I134="","",1440-I134)</f>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -5489,11 +5513,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5511,11 +5535,11 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J136" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K136" s="16"/>
@@ -5533,11 +5557,11 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J137" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K137" s="16"/>
@@ -5555,11 +5579,11 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J138" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K138" s="16"/>
@@ -5577,11 +5601,11 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J139" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K139" s="16"/>
@@ -5599,11 +5623,11 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J140" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K140" s="16"/>
@@ -5621,11 +5645,11 @@
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J141" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K141" s="16"/>
@@ -5643,11 +5667,11 @@
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J142" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K142" s="16"/>
@@ -5665,11 +5689,11 @@
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J143" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K143" s="16"/>
@@ -5687,11 +5711,11 @@
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J144" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K144" s="16"/>
@@ -5709,11 +5733,11 @@
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J145" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K145" s="16"/>
@@ -5731,11 +5755,11 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J146" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K146" s="16"/>
@@ -5753,11 +5777,11 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J147" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K147" s="16"/>
@@ -5775,11 +5799,11 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J148" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K148" s="16"/>
@@ -5797,11 +5821,11 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J149" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K149" s="16"/>
@@ -5819,11 +5843,11 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J150" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K150" s="16"/>
@@ -5841,11 +5865,11 @@
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
       <c r="I151" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J151" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K151" s="16"/>
@@ -5863,11 +5887,11 @@
       <c r="G152" s="14"/>
       <c r="H152" s="14"/>
       <c r="I152" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J152" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K152" s="16"/>
@@ -5885,11 +5909,11 @@
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J153" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K153" s="16"/>
@@ -5907,11 +5931,11 @@
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J154" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K154" s="16"/>
@@ -5929,11 +5953,11 @@
       <c r="G155" s="14"/>
       <c r="H155" s="14"/>
       <c r="I155" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J155" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K155" s="16"/>
@@ -5951,11 +5975,11 @@
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
       <c r="I156" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J156" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K156" s="16"/>
@@ -5973,11 +5997,11 @@
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J157" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K157" s="16"/>
@@ -5995,11 +6019,11 @@
       <c r="G158" s="14"/>
       <c r="H158" s="14"/>
       <c r="I158" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J158" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K158" s="16"/>
@@ -6017,11 +6041,11 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J159" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K159" s="16"/>
@@ -6039,11 +6063,11 @@
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
       <c r="I160" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J160" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K160" s="16"/>
@@ -6061,11 +6085,11 @@
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
       <c r="I161" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J161" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K161" s="16"/>
@@ -6083,11 +6107,11 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J162" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K162" s="16"/>
@@ -6105,11 +6129,11 @@
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
       <c r="I163" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J163" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K163" s="16"/>
@@ -6127,11 +6151,11 @@
       <c r="G164" s="14"/>
       <c r="H164" s="14"/>
       <c r="I164" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J164" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K164" s="16"/>
@@ -6149,11 +6173,11 @@
       <c r="G165" s="14"/>
       <c r="H165" s="14"/>
       <c r="I165" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J165" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K165" s="16"/>
@@ -6171,11 +6195,11 @@
       <c r="G166" s="14"/>
       <c r="H166" s="14"/>
       <c r="I166" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J166" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K166" s="16"/>
@@ -6193,11 +6217,11 @@
       <c r="G167" s="14"/>
       <c r="H167" s="14"/>
       <c r="I167" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J167" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K167" s="16"/>
@@ -6215,11 +6239,11 @@
       <c r="G168" s="14"/>
       <c r="H168" s="14"/>
       <c r="I168" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J168" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K168" s="16"/>
@@ -6237,11 +6261,11 @@
       <c r="G169" s="14"/>
       <c r="H169" s="14"/>
       <c r="I169" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J169" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K169" s="16"/>
@@ -6259,11 +6283,11 @@
       <c r="G170" s="14"/>
       <c r="H170" s="14"/>
       <c r="I170" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J170" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K170" s="16"/>
@@ -6281,11 +6305,11 @@
       <c r="G171" s="14"/>
       <c r="H171" s="14"/>
       <c r="I171" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J171" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K171" s="16"/>
@@ -6303,11 +6327,11 @@
       <c r="G172" s="14"/>
       <c r="H172" s="14"/>
       <c r="I172" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J172" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K172" s="16"/>
@@ -6325,11 +6349,11 @@
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
       <c r="I173" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J173" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K173" s="16"/>
@@ -6347,11 +6371,11 @@
       <c r="G174" s="14"/>
       <c r="H174" s="14"/>
       <c r="I174" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J174" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K174" s="16"/>
@@ -6369,11 +6393,11 @@
       <c r="G175" s="14"/>
       <c r="H175" s="14"/>
       <c r="I175" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J175" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K175" s="16"/>
@@ -6391,11 +6415,11 @@
       <c r="G176" s="14"/>
       <c r="H176" s="14"/>
       <c r="I176" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J176" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K176" s="16"/>
@@ -6413,11 +6437,11 @@
       <c r="G177" s="14"/>
       <c r="H177" s="14"/>
       <c r="I177" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J177" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K177" s="16"/>
@@ -6435,11 +6459,11 @@
       <c r="G178" s="14"/>
       <c r="H178" s="14"/>
       <c r="I178" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J178" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K178" s="16"/>
@@ -6457,11 +6481,11 @@
       <c r="G179" s="14"/>
       <c r="H179" s="14"/>
       <c r="I179" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J179" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K179" s="16"/>
@@ -6479,11 +6503,11 @@
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
       <c r="I180" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J180" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K180" s="16"/>
@@ -6501,11 +6525,11 @@
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J181" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K181" s="16"/>
@@ -6523,11 +6547,11 @@
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J182" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K182" s="16"/>
@@ -6545,11 +6569,11 @@
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J183" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K183" s="16"/>
@@ -6567,11 +6591,11 @@
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
       <c r="I184" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J184" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K184" s="16"/>
@@ -6589,11 +6613,11 @@
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
       <c r="I185" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J185" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K185" s="16"/>
@@ -6611,11 +6635,11 @@
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J186" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K186" s="16"/>
@@ -6633,11 +6657,11 @@
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J187" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K187" s="16"/>
@@ -6655,11 +6679,11 @@
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
       <c r="I188" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J188" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K188" s="16"/>
@@ -6677,11 +6701,11 @@
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
       <c r="I189" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J189" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K189" s="16"/>
@@ -6699,11 +6723,11 @@
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J190" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K190" s="16"/>
@@ -6721,11 +6745,11 @@
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J191" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K191" s="16"/>
@@ -6743,11 +6767,11 @@
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J192" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K192" s="16"/>
@@ -6765,11 +6789,11 @@
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
       <c r="I193" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J193" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K193" s="16"/>
@@ -6787,11 +6811,11 @@
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
       <c r="I194" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J194" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K194" s="16"/>
@@ -6809,11 +6833,11 @@
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J195" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K195" s="16"/>
@@ -6831,11 +6855,11 @@
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J196" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K196" s="16"/>
@@ -6853,11 +6877,11 @@
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J197" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K197" s="16"/>
@@ -6875,11 +6899,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="8">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" ref="I198:I261" si="10">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="9">IF(I198="","",1440-I198)</f>
+        <f t="shared" ref="J198:J261" si="11">IF(I198="","",1440-I198)</f>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -6897,11 +6921,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -6919,11 +6943,11 @@
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J200" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K200" s="16"/>
@@ -6941,11 +6965,11 @@
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
       <c r="I201" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J201" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K201" s="16"/>
@@ -6963,11 +6987,11 @@
       <c r="G202" s="14"/>
       <c r="H202" s="14"/>
       <c r="I202" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J202" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K202" s="16"/>
@@ -6985,11 +7009,11 @@
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
       <c r="I203" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J203" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K203" s="16"/>
@@ -7007,11 +7031,11 @@
       <c r="G204" s="14"/>
       <c r="H204" s="14"/>
       <c r="I204" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J204" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K204" s="16"/>
@@ -7029,11 +7053,11 @@
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J205" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K205" s="16"/>
@@ -7051,11 +7075,11 @@
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J206" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K206" s="16"/>
@@ -7073,11 +7097,11 @@
       <c r="G207" s="14"/>
       <c r="H207" s="14"/>
       <c r="I207" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J207" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K207" s="16"/>
@@ -7095,11 +7119,11 @@
       <c r="G208" s="14"/>
       <c r="H208" s="14"/>
       <c r="I208" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J208" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K208" s="16"/>
@@ -7117,11 +7141,11 @@
       <c r="G209" s="14"/>
       <c r="H209" s="14"/>
       <c r="I209" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J209" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K209" s="16"/>
@@ -7139,11 +7163,11 @@
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J210" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K210" s="16"/>
@@ -7161,11 +7185,11 @@
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J211" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K211" s="16"/>
@@ -7183,11 +7207,11 @@
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J212" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K212" s="16"/>
@@ -7205,11 +7229,11 @@
       <c r="G213" s="14"/>
       <c r="H213" s="14"/>
       <c r="I213" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J213" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K213" s="16"/>
@@ -7227,11 +7251,11 @@
       <c r="G214" s="14"/>
       <c r="H214" s="14"/>
       <c r="I214" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J214" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K214" s="16"/>
@@ -7249,11 +7273,11 @@
       <c r="G215" s="14"/>
       <c r="H215" s="14"/>
       <c r="I215" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J215" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K215" s="16"/>
@@ -7271,11 +7295,11 @@
       <c r="G216" s="14"/>
       <c r="H216" s="14"/>
       <c r="I216" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J216" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K216" s="16"/>
@@ -7293,11 +7317,11 @@
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J217" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K217" s="16"/>
@@ -7315,11 +7339,11 @@
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J218" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K218" s="16"/>
@@ -7337,11 +7361,11 @@
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J219" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K219" s="16"/>
@@ -7359,11 +7383,11 @@
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J220" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K220" s="16"/>
@@ -7381,11 +7405,11 @@
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J221" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K221" s="16"/>
@@ -7403,11 +7427,11 @@
       <c r="G222" s="14"/>
       <c r="H222" s="14"/>
       <c r="I222" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J222" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K222" s="16"/>
@@ -7425,11 +7449,11 @@
       <c r="G223" s="14"/>
       <c r="H223" s="14"/>
       <c r="I223" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J223" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K223" s="16"/>
@@ -7447,11 +7471,11 @@
       <c r="G224" s="14"/>
       <c r="H224" s="14"/>
       <c r="I224" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J224" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K224" s="16"/>
@@ -7469,11 +7493,11 @@
       <c r="G225" s="14"/>
       <c r="H225" s="14"/>
       <c r="I225" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J225" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K225" s="16"/>
@@ -7491,11 +7515,11 @@
       <c r="G226" s="14"/>
       <c r="H226" s="14"/>
       <c r="I226" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J226" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K226" s="16"/>
@@ -7513,11 +7537,11 @@
       <c r="G227" s="14"/>
       <c r="H227" s="14"/>
       <c r="I227" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J227" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K227" s="16"/>
@@ -7535,11 +7559,11 @@
       <c r="G228" s="14"/>
       <c r="H228" s="14"/>
       <c r="I228" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J228" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K228" s="16"/>
@@ -7557,11 +7581,11 @@
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J229" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K229" s="16"/>
@@ -7579,11 +7603,11 @@
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J230" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K230" s="16"/>
@@ -7601,11 +7625,11 @@
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
       <c r="I231" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J231" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K231" s="16"/>
@@ -7623,11 +7647,11 @@
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
       <c r="I232" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J232" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K232" s="16"/>
@@ -7645,11 +7669,11 @@
       <c r="G233" s="14"/>
       <c r="H233" s="14"/>
       <c r="I233" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J233" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K233" s="16"/>
@@ -7667,11 +7691,11 @@
       <c r="G234" s="14"/>
       <c r="H234" s="14"/>
       <c r="I234" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J234" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K234" s="16"/>
@@ -7689,11 +7713,11 @@
       <c r="G235" s="14"/>
       <c r="H235" s="14"/>
       <c r="I235" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J235" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K235" s="16"/>
@@ -7711,11 +7735,11 @@
       <c r="G236" s="14"/>
       <c r="H236" s="14"/>
       <c r="I236" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J236" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K236" s="16"/>
@@ -7733,11 +7757,11 @@
       <c r="G237" s="14"/>
       <c r="H237" s="14"/>
       <c r="I237" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J237" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K237" s="16"/>
@@ -7755,11 +7779,11 @@
       <c r="G238" s="14"/>
       <c r="H238" s="14"/>
       <c r="I238" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J238" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K238" s="16"/>
@@ -7777,11 +7801,11 @@
       <c r="G239" s="14"/>
       <c r="H239" s="14"/>
       <c r="I239" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J239" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K239" s="16"/>
@@ -7799,11 +7823,11 @@
       <c r="G240" s="14"/>
       <c r="H240" s="14"/>
       <c r="I240" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J240" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K240" s="16"/>
@@ -7821,11 +7845,11 @@
       <c r="G241" s="14"/>
       <c r="H241" s="14"/>
       <c r="I241" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J241" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K241" s="16"/>
@@ -7843,11 +7867,11 @@
       <c r="G242" s="14"/>
       <c r="H242" s="14"/>
       <c r="I242" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J242" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K242" s="16"/>
@@ -7865,11 +7889,11 @@
       <c r="G243" s="14"/>
       <c r="H243" s="14"/>
       <c r="I243" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J243" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K243" s="16"/>
@@ -7887,11 +7911,11 @@
       <c r="G244" s="14"/>
       <c r="H244" s="14"/>
       <c r="I244" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J244" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K244" s="16"/>
@@ -7909,11 +7933,11 @@
       <c r="G245" s="14"/>
       <c r="H245" s="14"/>
       <c r="I245" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J245" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K245" s="16"/>
@@ -7931,11 +7955,11 @@
       <c r="G246" s="14"/>
       <c r="H246" s="14"/>
       <c r="I246" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J246" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K246" s="16"/>
@@ -7953,11 +7977,11 @@
       <c r="G247" s="14"/>
       <c r="H247" s="14"/>
       <c r="I247" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J247" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K247" s="16"/>
@@ -7975,11 +7999,11 @@
       <c r="G248" s="14"/>
       <c r="H248" s="14"/>
       <c r="I248" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J248" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K248" s="16"/>
@@ -7997,11 +8021,11 @@
       <c r="G249" s="14"/>
       <c r="H249" s="14"/>
       <c r="I249" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J249" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K249" s="16"/>
@@ -8019,11 +8043,11 @@
       <c r="G250" s="14"/>
       <c r="H250" s="14"/>
       <c r="I250" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J250" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K250" s="16"/>
@@ -8041,11 +8065,11 @@
       <c r="G251" s="14"/>
       <c r="H251" s="14"/>
       <c r="I251" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J251" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K251" s="16"/>
@@ -8063,11 +8087,11 @@
       <c r="G252" s="14"/>
       <c r="H252" s="14"/>
       <c r="I252" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J252" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K252" s="16"/>
@@ -8085,11 +8109,11 @@
       <c r="G253" s="14"/>
       <c r="H253" s="14"/>
       <c r="I253" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J253" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K253" s="16"/>
@@ -8107,11 +8131,11 @@
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
       <c r="I254" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J254" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K254" s="16"/>
@@ -8129,11 +8153,11 @@
       <c r="G255" s="14"/>
       <c r="H255" s="14"/>
       <c r="I255" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J255" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K255" s="16"/>
@@ -8151,11 +8175,11 @@
       <c r="G256" s="14"/>
       <c r="H256" s="14"/>
       <c r="I256" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J256" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K256" s="16"/>
@@ -8173,11 +8197,11 @@
       <c r="G257" s="14"/>
       <c r="H257" s="14"/>
       <c r="I257" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J257" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K257" s="16"/>
@@ -8195,11 +8219,11 @@
       <c r="G258" s="14"/>
       <c r="H258" s="14"/>
       <c r="I258" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J258" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K258" s="16"/>
@@ -8217,11 +8241,11 @@
       <c r="G259" s="14"/>
       <c r="H259" s="14"/>
       <c r="I259" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J259" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K259" s="16"/>
@@ -8239,11 +8263,11 @@
       <c r="G260" s="14"/>
       <c r="H260" s="14"/>
       <c r="I260" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J260" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K260" s="16"/>
@@ -8261,11 +8285,11 @@
       <c r="G261" s="14"/>
       <c r="H261" s="14"/>
       <c r="I261" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J261" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K261" s="16"/>
@@ -8283,11 +8307,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="10">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" ref="I262:I325" si="12">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="11">IF(I262="","",1440-I262)</f>
+        <f t="shared" ref="J262:J325" si="13">IF(I262="","",1440-I262)</f>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -8305,11 +8329,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8327,11 +8351,11 @@
       <c r="G264" s="14"/>
       <c r="H264" s="14"/>
       <c r="I264" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J264" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K264" s="16"/>
@@ -8349,11 +8373,11 @@
       <c r="G265" s="14"/>
       <c r="H265" s="14"/>
       <c r="I265" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J265" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K265" s="16"/>
@@ -8371,11 +8395,11 @@
       <c r="G266" s="14"/>
       <c r="H266" s="14"/>
       <c r="I266" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J266" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K266" s="16"/>
@@ -8393,11 +8417,11 @@
       <c r="G267" s="14"/>
       <c r="H267" s="14"/>
       <c r="I267" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J267" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K267" s="16"/>
@@ -8415,11 +8439,11 @@
       <c r="G268" s="14"/>
       <c r="H268" s="14"/>
       <c r="I268" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J268" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K268" s="16"/>
@@ -8437,11 +8461,11 @@
       <c r="G269" s="14"/>
       <c r="H269" s="14"/>
       <c r="I269" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J269" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K269" s="16"/>
@@ -8459,11 +8483,11 @@
       <c r="G270" s="14"/>
       <c r="H270" s="14"/>
       <c r="I270" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J270" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K270" s="16"/>
@@ -8481,11 +8505,11 @@
       <c r="G271" s="14"/>
       <c r="H271" s="14"/>
       <c r="I271" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J271" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K271" s="16"/>
@@ -8503,11 +8527,11 @@
       <c r="G272" s="14"/>
       <c r="H272" s="14"/>
       <c r="I272" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J272" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K272" s="16"/>
@@ -8525,11 +8549,11 @@
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
       <c r="I273" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J273" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K273" s="16"/>
@@ -8547,11 +8571,11 @@
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
       <c r="I274" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J274" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K274" s="16"/>
@@ -8569,11 +8593,11 @@
       <c r="G275" s="14"/>
       <c r="H275" s="14"/>
       <c r="I275" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J275" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K275" s="16"/>
@@ -8591,11 +8615,11 @@
       <c r="G276" s="14"/>
       <c r="H276" s="14"/>
       <c r="I276" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J276" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K276" s="16"/>
@@ -8613,11 +8637,11 @@
       <c r="G277" s="14"/>
       <c r="H277" s="14"/>
       <c r="I277" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J277" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K277" s="16"/>
@@ -8635,11 +8659,11 @@
       <c r="G278" s="14"/>
       <c r="H278" s="14"/>
       <c r="I278" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J278" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K278" s="16"/>
@@ -8657,11 +8681,11 @@
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
       <c r="I279" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J279" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K279" s="16"/>
@@ -8679,11 +8703,11 @@
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
       <c r="I280" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J280" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K280" s="16"/>
@@ -8701,11 +8725,11 @@
       <c r="G281" s="14"/>
       <c r="H281" s="14"/>
       <c r="I281" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J281" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K281" s="16"/>
@@ -8723,11 +8747,11 @@
       <c r="G282" s="14"/>
       <c r="H282" s="14"/>
       <c r="I282" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J282" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K282" s="16"/>
@@ -8745,11 +8769,11 @@
       <c r="G283" s="14"/>
       <c r="H283" s="14"/>
       <c r="I283" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J283" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K283" s="16"/>
@@ -8767,11 +8791,11 @@
       <c r="G284" s="14"/>
       <c r="H284" s="14"/>
       <c r="I284" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J284" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K284" s="16"/>
@@ -8789,11 +8813,11 @@
       <c r="G285" s="14"/>
       <c r="H285" s="14"/>
       <c r="I285" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J285" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K285" s="16"/>
@@ -8811,11 +8835,11 @@
       <c r="G286" s="14"/>
       <c r="H286" s="14"/>
       <c r="I286" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J286" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K286" s="16"/>
@@ -8833,11 +8857,11 @@
       <c r="G287" s="14"/>
       <c r="H287" s="14"/>
       <c r="I287" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J287" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K287" s="16"/>
@@ -8855,11 +8879,11 @@
       <c r="G288" s="14"/>
       <c r="H288" s="14"/>
       <c r="I288" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J288" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K288" s="16"/>
@@ -8877,11 +8901,11 @@
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
       <c r="I289" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J289" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K289" s="16"/>
@@ -8899,11 +8923,11 @@
       <c r="G290" s="14"/>
       <c r="H290" s="14"/>
       <c r="I290" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J290" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K290" s="16"/>
@@ -8921,11 +8945,11 @@
       <c r="G291" s="14"/>
       <c r="H291" s="14"/>
       <c r="I291" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J291" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K291" s="16"/>
@@ -8943,11 +8967,11 @@
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
       <c r="I292" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J292" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K292" s="16"/>
@@ -8965,11 +8989,11 @@
       <c r="G293" s="14"/>
       <c r="H293" s="14"/>
       <c r="I293" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J293" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K293" s="16"/>
@@ -8987,11 +9011,11 @@
       <c r="G294" s="14"/>
       <c r="H294" s="14"/>
       <c r="I294" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J294" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K294" s="16"/>
@@ -9009,11 +9033,11 @@
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
       <c r="I295" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J295" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K295" s="16"/>
@@ -9031,11 +9055,11 @@
       <c r="G296" s="14"/>
       <c r="H296" s="14"/>
       <c r="I296" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J296" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K296" s="16"/>
@@ -9053,11 +9077,11 @@
       <c r="G297" s="14"/>
       <c r="H297" s="14"/>
       <c r="I297" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J297" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K297" s="16"/>
@@ -9075,11 +9099,11 @@
       <c r="G298" s="14"/>
       <c r="H298" s="14"/>
       <c r="I298" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J298" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K298" s="16"/>
@@ -9097,11 +9121,11 @@
       <c r="G299" s="14"/>
       <c r="H299" s="14"/>
       <c r="I299" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J299" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K299" s="16"/>
@@ -9119,11 +9143,11 @@
       <c r="G300" s="14"/>
       <c r="H300" s="14"/>
       <c r="I300" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J300" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K300" s="16"/>
@@ -9141,11 +9165,11 @@
       <c r="G301" s="14"/>
       <c r="H301" s="14"/>
       <c r="I301" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J301" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K301" s="16"/>
@@ -9163,11 +9187,11 @@
       <c r="G302" s="14"/>
       <c r="H302" s="14"/>
       <c r="I302" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J302" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K302" s="16"/>
@@ -9185,11 +9209,11 @@
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
       <c r="I303" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J303" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K303" s="16"/>
@@ -9207,11 +9231,11 @@
       <c r="G304" s="14"/>
       <c r="H304" s="14"/>
       <c r="I304" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J304" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K304" s="16"/>
@@ -9229,11 +9253,11 @@
       <c r="G305" s="14"/>
       <c r="H305" s="14"/>
       <c r="I305" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J305" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K305" s="16"/>
@@ -9251,11 +9275,11 @@
       <c r="G306" s="14"/>
       <c r="H306" s="14"/>
       <c r="I306" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J306" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K306" s="16"/>
@@ -9273,11 +9297,11 @@
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
       <c r="I307" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J307" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K307" s="16"/>
@@ -9295,11 +9319,11 @@
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
       <c r="I308" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J308" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K308" s="16"/>
@@ -9317,11 +9341,11 @@
       <c r="G309" s="14"/>
       <c r="H309" s="14"/>
       <c r="I309" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J309" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K309" s="16"/>
@@ -9339,11 +9363,11 @@
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
       <c r="I310" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J310" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K310" s="16"/>
@@ -9361,11 +9385,11 @@
       <c r="G311" s="14"/>
       <c r="H311" s="14"/>
       <c r="I311" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J311" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K311" s="16"/>
@@ -9383,11 +9407,11 @@
       <c r="G312" s="14"/>
       <c r="H312" s="14"/>
       <c r="I312" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J312" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K312" s="16"/>
@@ -9405,11 +9429,11 @@
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
       <c r="I313" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J313" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K313" s="16"/>
@@ -9427,11 +9451,11 @@
       <c r="G314" s="14"/>
       <c r="H314" s="14"/>
       <c r="I314" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J314" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K314" s="16"/>
@@ -9449,11 +9473,11 @@
       <c r="G315" s="14"/>
       <c r="H315" s="14"/>
       <c r="I315" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J315" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K315" s="16"/>
@@ -9471,11 +9495,11 @@
       <c r="G316" s="14"/>
       <c r="H316" s="14"/>
       <c r="I316" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J316" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K316" s="16"/>
@@ -9493,11 +9517,11 @@
       <c r="G317" s="14"/>
       <c r="H317" s="14"/>
       <c r="I317" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J317" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K317" s="16"/>
@@ -9515,11 +9539,11 @@
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
       <c r="I318" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J318" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K318" s="16"/>
@@ -9537,11 +9561,11 @@
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
       <c r="I319" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J319" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K319" s="16"/>
@@ -9559,11 +9583,11 @@
       <c r="G320" s="14"/>
       <c r="H320" s="14"/>
       <c r="I320" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J320" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K320" s="16"/>
@@ -9581,11 +9605,11 @@
       <c r="G321" s="14"/>
       <c r="H321" s="14"/>
       <c r="I321" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J321" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K321" s="16"/>
@@ -9603,11 +9627,11 @@
       <c r="G322" s="14"/>
       <c r="H322" s="14"/>
       <c r="I322" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J322" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K322" s="16"/>
@@ -9625,11 +9649,11 @@
       <c r="G323" s="14"/>
       <c r="H323" s="14"/>
       <c r="I323" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J323" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K323" s="16"/>
@@ -9647,11 +9671,11 @@
       <c r="G324" s="14"/>
       <c r="H324" s="14"/>
       <c r="I324" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J324" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K324" s="16"/>
@@ -9669,11 +9693,11 @@
       <c r="G325" s="14"/>
       <c r="H325" s="14"/>
       <c r="I325" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J325" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K325" s="16"/>
@@ -9691,11 +9715,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="12">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" ref="I326:I389" si="14">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="13">IF(I326="","",1440-I326)</f>
+        <f t="shared" ref="J326:J389" si="15">IF(I326="","",1440-I326)</f>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -9713,11 +9737,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -9735,11 +9759,11 @@
       <c r="G328" s="14"/>
       <c r="H328" s="14"/>
       <c r="I328" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J328" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K328" s="16"/>
@@ -9757,11 +9781,11 @@
       <c r="G329" s="14"/>
       <c r="H329" s="14"/>
       <c r="I329" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J329" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K329" s="16"/>
@@ -9779,11 +9803,11 @@
       <c r="G330" s="14"/>
       <c r="H330" s="14"/>
       <c r="I330" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J330" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K330" s="16"/>
@@ -9801,11 +9825,11 @@
       <c r="G331" s="14"/>
       <c r="H331" s="14"/>
       <c r="I331" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J331" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K331" s="16"/>
@@ -9823,11 +9847,11 @@
       <c r="G332" s="14"/>
       <c r="H332" s="14"/>
       <c r="I332" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J332" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K332" s="16"/>
@@ -9845,11 +9869,11 @@
       <c r="G333" s="14"/>
       <c r="H333" s="14"/>
       <c r="I333" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J333" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K333" s="16"/>
@@ -9867,11 +9891,11 @@
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
       <c r="I334" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J334" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K334" s="16"/>
@@ -9889,11 +9913,11 @@
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
       <c r="I335" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J335" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K335" s="16"/>
@@ -9911,11 +9935,11 @@
       <c r="G336" s="14"/>
       <c r="H336" s="14"/>
       <c r="I336" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J336" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K336" s="16"/>
@@ -9933,11 +9957,11 @@
       <c r="G337" s="14"/>
       <c r="H337" s="14"/>
       <c r="I337" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J337" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K337" s="16"/>
@@ -9955,11 +9979,11 @@
       <c r="G338" s="14"/>
       <c r="H338" s="14"/>
       <c r="I338" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J338" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K338" s="16"/>
@@ -9977,11 +10001,11 @@
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
       <c r="I339" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J339" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K339" s="16"/>
@@ -9999,11 +10023,11 @@
       <c r="G340" s="14"/>
       <c r="H340" s="14"/>
       <c r="I340" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J340" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K340" s="16"/>
@@ -10021,11 +10045,11 @@
       <c r="G341" s="14"/>
       <c r="H341" s="14"/>
       <c r="I341" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J341" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K341" s="16"/>
@@ -10043,11 +10067,11 @@
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
       <c r="I342" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J342" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K342" s="16"/>
@@ -10065,11 +10089,11 @@
       <c r="G343" s="14"/>
       <c r="H343" s="14"/>
       <c r="I343" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J343" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K343" s="16"/>
@@ -10087,11 +10111,11 @@
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
       <c r="I344" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J344" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K344" s="16"/>
@@ -10109,11 +10133,11 @@
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
       <c r="I345" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J345" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K345" s="16"/>
@@ -10131,11 +10155,11 @@
       <c r="G346" s="14"/>
       <c r="H346" s="14"/>
       <c r="I346" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J346" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K346" s="16"/>
@@ -10153,11 +10177,11 @@
       <c r="G347" s="14"/>
       <c r="H347" s="14"/>
       <c r="I347" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J347" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K347" s="16"/>
@@ -10175,11 +10199,11 @@
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
       <c r="I348" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J348" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K348" s="16"/>
@@ -10197,11 +10221,11 @@
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
       <c r="I349" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J349" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K349" s="16"/>
@@ -10219,11 +10243,11 @@
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
       <c r="I350" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J350" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K350" s="16"/>
@@ -10241,11 +10265,11 @@
       <c r="G351" s="14"/>
       <c r="H351" s="14"/>
       <c r="I351" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J351" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K351" s="16"/>
@@ -10263,11 +10287,11 @@
       <c r="G352" s="14"/>
       <c r="H352" s="14"/>
       <c r="I352" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J352" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K352" s="16"/>
@@ -10285,11 +10309,11 @@
       <c r="G353" s="14"/>
       <c r="H353" s="14"/>
       <c r="I353" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J353" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K353" s="16"/>
@@ -10307,11 +10331,11 @@
       <c r="G354" s="14"/>
       <c r="H354" s="14"/>
       <c r="I354" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J354" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K354" s="16"/>
@@ -10329,11 +10353,11 @@
       <c r="G355" s="14"/>
       <c r="H355" s="14"/>
       <c r="I355" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J355" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K355" s="16"/>
@@ -10351,11 +10375,11 @@
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
       <c r="I356" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J356" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K356" s="16"/>
@@ -10373,11 +10397,11 @@
       <c r="G357" s="14"/>
       <c r="H357" s="14"/>
       <c r="I357" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J357" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K357" s="16"/>
@@ -10395,11 +10419,11 @@
       <c r="G358" s="14"/>
       <c r="H358" s="14"/>
       <c r="I358" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J358" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K358" s="16"/>
@@ -10417,11 +10441,11 @@
       <c r="G359" s="14"/>
       <c r="H359" s="14"/>
       <c r="I359" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J359" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K359" s="16"/>
@@ -10439,11 +10463,11 @@
       <c r="G360" s="14"/>
       <c r="H360" s="14"/>
       <c r="I360" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J360" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K360" s="16"/>
@@ -10461,11 +10485,11 @@
       <c r="G361" s="14"/>
       <c r="H361" s="14"/>
       <c r="I361" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J361" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K361" s="16"/>
@@ -10483,11 +10507,11 @@
       <c r="G362" s="14"/>
       <c r="H362" s="14"/>
       <c r="I362" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J362" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K362" s="16"/>
@@ -10505,11 +10529,11 @@
       <c r="G363" s="14"/>
       <c r="H363" s="14"/>
       <c r="I363" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J363" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K363" s="16"/>
@@ -10527,11 +10551,11 @@
       <c r="G364" s="14"/>
       <c r="H364" s="14"/>
       <c r="I364" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J364" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K364" s="16"/>
@@ -10549,11 +10573,11 @@
       <c r="G365" s="14"/>
       <c r="H365" s="14"/>
       <c r="I365" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J365" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K365" s="16"/>
@@ -10571,11 +10595,11 @@
       <c r="G366" s="14"/>
       <c r="H366" s="14"/>
       <c r="I366" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J366" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K366" s="16"/>
@@ -10593,11 +10617,11 @@
       <c r="G367" s="14"/>
       <c r="H367" s="14"/>
       <c r="I367" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J367" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K367" s="16"/>
@@ -10615,11 +10639,11 @@
       <c r="G368" s="14"/>
       <c r="H368" s="14"/>
       <c r="I368" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J368" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K368" s="16"/>
@@ -10637,11 +10661,11 @@
       <c r="G369" s="14"/>
       <c r="H369" s="14"/>
       <c r="I369" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J369" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K369" s="16"/>
@@ -10659,11 +10683,11 @@
       <c r="G370" s="14"/>
       <c r="H370" s="14"/>
       <c r="I370" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J370" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K370" s="16"/>
@@ -10681,11 +10705,11 @@
       <c r="G371" s="14"/>
       <c r="H371" s="14"/>
       <c r="I371" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J371" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K371" s="16"/>
@@ -10703,11 +10727,11 @@
       <c r="G372" s="14"/>
       <c r="H372" s="14"/>
       <c r="I372" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J372" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K372" s="16"/>
@@ -10725,11 +10749,11 @@
       <c r="G373" s="14"/>
       <c r="H373" s="14"/>
       <c r="I373" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J373" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K373" s="16"/>
@@ -10747,11 +10771,11 @@
       <c r="G374" s="14"/>
       <c r="H374" s="14"/>
       <c r="I374" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J374" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K374" s="16"/>
@@ -10769,11 +10793,11 @@
       <c r="G375" s="14"/>
       <c r="H375" s="14"/>
       <c r="I375" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J375" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K375" s="16"/>
@@ -10791,11 +10815,11 @@
       <c r="G376" s="14"/>
       <c r="H376" s="14"/>
       <c r="I376" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J376" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K376" s="16"/>
@@ -10813,11 +10837,11 @@
       <c r="G377" s="14"/>
       <c r="H377" s="14"/>
       <c r="I377" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J377" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K377" s="16"/>
@@ -10835,11 +10859,11 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K378" s="16"/>
@@ -10857,11 +10881,11 @@
       <c r="G379" s="14"/>
       <c r="H379" s="14"/>
       <c r="I379" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J379" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K379" s="16"/>
@@ -10879,11 +10903,11 @@
       <c r="G380" s="14"/>
       <c r="H380" s="14"/>
       <c r="I380" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J380" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K380" s="16"/>
@@ -10901,11 +10925,11 @@
       <c r="G381" s="14"/>
       <c r="H381" s="14"/>
       <c r="I381" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J381" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K381" s="16"/>
@@ -10923,11 +10947,11 @@
       <c r="G382" s="14"/>
       <c r="H382" s="14"/>
       <c r="I382" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J382" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K382" s="16"/>
@@ -10945,11 +10969,11 @@
       <c r="G383" s="14"/>
       <c r="H383" s="14"/>
       <c r="I383" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J383" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K383" s="16"/>
@@ -10967,11 +10991,11 @@
       <c r="G384" s="14"/>
       <c r="H384" s="14"/>
       <c r="I384" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J384" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K384" s="16"/>
@@ -10989,11 +11013,11 @@
       <c r="G385" s="14"/>
       <c r="H385" s="14"/>
       <c r="I385" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J385" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K385" s="16"/>
@@ -11011,11 +11035,11 @@
       <c r="G386" s="14"/>
       <c r="H386" s="14"/>
       <c r="I386" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J386" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K386" s="16"/>
@@ -11033,11 +11057,11 @@
       <c r="G387" s="14"/>
       <c r="H387" s="14"/>
       <c r="I387" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J387" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K387" s="16"/>
@@ -11055,11 +11079,11 @@
       <c r="G388" s="14"/>
       <c r="H388" s="14"/>
       <c r="I388" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J388" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K388" s="16"/>
@@ -11077,11 +11101,11 @@
       <c r="G389" s="14"/>
       <c r="H389" s="14"/>
       <c r="I389" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J389" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K389" s="16"/>
@@ -11099,11 +11123,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="14">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="16">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="15">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="17">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -11121,11 +11145,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -11143,11 +11167,11 @@
       <c r="G392" s="14"/>
       <c r="H392" s="14"/>
       <c r="I392" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J392" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K392" s="16"/>
@@ -11165,11 +11189,11 @@
       <c r="G393" s="14"/>
       <c r="H393" s="14"/>
       <c r="I393" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J393" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K393" s="16"/>
@@ -11187,11 +11211,11 @@
       <c r="G394" s="14"/>
       <c r="H394" s="14"/>
       <c r="I394" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J394" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K394" s="16"/>
@@ -11209,11 +11233,11 @@
       <c r="G395" s="14"/>
       <c r="H395" s="14"/>
       <c r="I395" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J395" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K395" s="16"/>
@@ -11231,11 +11255,11 @@
       <c r="G396" s="14"/>
       <c r="H396" s="14"/>
       <c r="I396" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J396" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K396" s="16"/>
@@ -11253,11 +11277,11 @@
       <c r="G397" s="14"/>
       <c r="H397" s="14"/>
       <c r="I397" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J397" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K397" s="16"/>
@@ -11275,11 +11299,11 @@
       <c r="G398" s="14"/>
       <c r="H398" s="14"/>
       <c r="I398" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J398" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K398" s="16"/>
@@ -11297,11 +11321,11 @@
       <c r="G399" s="14"/>
       <c r="H399" s="14"/>
       <c r="I399" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J399" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K399" s="16"/>
@@ -11319,11 +11343,11 @@
       <c r="G400" s="14"/>
       <c r="H400" s="14"/>
       <c r="I400" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J400" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K400" s="16"/>
@@ -11341,11 +11365,11 @@
       <c r="G401" s="14"/>
       <c r="H401" s="14"/>
       <c r="I401" s="15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="J401" s="15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="K401" s="16"/>

</xml_diff>

<commit_message>
UPdate of 11, 12 and 13th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="131">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -422,6 +422,15 @@
   </si>
   <si>
     <t>College Leave</t>
+  </si>
+  <si>
+    <t>Mid term Exam</t>
+  </si>
+  <si>
+    <t>Data Networking Mid term Exam</t>
+  </si>
+  <si>
+    <t>Object Oriented Programming Using C++  Mid term Exam</t>
   </si>
 </sst>
 </file>
@@ -4008,70 +4017,142 @@
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="14"/>
-      <c r="F67" s="14"/>
-      <c r="G67" s="14"/>
-      <c r="H67" s="14"/>
-      <c r="I67" s="15" t="str">
+      <c r="A67" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B67" s="14">
+        <v>360</v>
+      </c>
+      <c r="C67" s="14">
+        <v>30</v>
+      </c>
+      <c r="D67" s="14">
+        <v>300</v>
+      </c>
+      <c r="E67" s="14">
+        <v>30</v>
+      </c>
+      <c r="F67" s="14">
+        <v>0</v>
+      </c>
+      <c r="G67" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H67" s="14">
+        <v>100</v>
+      </c>
+      <c r="I67" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="15" t="str">
+        <v>820</v>
+      </c>
+      <c r="J67" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
-      <c r="N67" s="17"/>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A68" s="13"/>
-      <c r="B68" s="14"/>
-      <c r="C68" s="14"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="14"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="14"/>
-      <c r="H68" s="14"/>
-      <c r="I68" s="15" t="str">
+        <v>620</v>
+      </c>
+      <c r="K67" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L67" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M67" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N67" s="17" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A68" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B68" s="14">
+        <v>360</v>
+      </c>
+      <c r="C68" s="14">
+        <v>30</v>
+      </c>
+      <c r="D68" s="14">
+        <v>300</v>
+      </c>
+      <c r="E68" s="14">
+        <v>60</v>
+      </c>
+      <c r="F68" s="14">
+        <v>0</v>
+      </c>
+      <c r="G68" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="H68" s="14">
+        <v>60</v>
+      </c>
+      <c r="I68" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="15" t="str">
+        <v>810</v>
+      </c>
+      <c r="J68" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
-      <c r="N68" s="17"/>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="13"/>
-      <c r="B69" s="14"/>
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
-      <c r="G69" s="14"/>
-      <c r="H69" s="14"/>
-      <c r="I69" s="15" t="str">
+        <v>630</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L68" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="M68" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="N68" s="17" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A69" s="13">
+        <v>46308</v>
+      </c>
+      <c r="B69" s="14">
+        <v>360</v>
+      </c>
+      <c r="C69" s="14">
+        <v>30</v>
+      </c>
+      <c r="D69" s="14">
+        <v>300</v>
+      </c>
+      <c r="E69" s="14">
+        <v>60</v>
+      </c>
+      <c r="F69" s="14">
+        <v>0</v>
+      </c>
+      <c r="G69" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="H69" s="14">
+        <v>60</v>
+      </c>
+      <c r="I69" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="15" t="str">
+        <v>810</v>
+      </c>
+      <c r="J69" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
-      <c r="N69" s="17"/>
+        <v>630</v>
+      </c>
+      <c r="K69" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="M69" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N69" s="17" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="13"/>

</xml_diff>

<commit_message>
Update of 14th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="132">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -431,6 +431,9 @@
   </si>
   <si>
     <t>Object Oriented Programming Using C++  Mid term Exam</t>
+  </si>
+  <si>
+    <t>Adavanced Database Techniques Mid term Exam</t>
   </si>
 </sst>
 </file>
@@ -4154,27 +4157,51 @@
         <v>130</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A70" s="13"/>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="14"/>
-      <c r="H70" s="14"/>
-      <c r="I70" s="15" t="str">
+    <row r="70" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A70" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B70" s="14">
+        <v>450</v>
+      </c>
+      <c r="C70" s="14">
+        <v>60</v>
+      </c>
+      <c r="D70" s="14">
+        <v>300</v>
+      </c>
+      <c r="E70" s="14">
+        <v>0</v>
+      </c>
+      <c r="F70" s="14">
+        <v>0</v>
+      </c>
+      <c r="G70" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="H70" s="14">
+        <v>60</v>
+      </c>
+      <c r="I70" s="15">
         <f t="shared" ref="I70:I133" si="6">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v/>
-      </c>
-      <c r="J70" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J70" s="15">
         <f t="shared" ref="J70:J133" si="7">IF(I70="","",1440-I70)</f>
-        <v/>
-      </c>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-      <c r="N70" s="17"/>
+        <v>570</v>
+      </c>
+      <c r="K70" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="M70" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="N70" s="17" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>

</xml_diff>

<commit_message>
Update 15th, 16th, 17th, 18th and 19th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="138">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -434,6 +434,24 @@
   </si>
   <si>
     <t>Adavanced Database Techniques Mid term Exam</t>
+  </si>
+  <si>
+    <t>Analytical Skills - 1 Mid term Exam</t>
+  </si>
+  <si>
+    <t>Upper Internediate Communication Skills Mid term Exam</t>
+  </si>
+  <si>
+    <t>Preparataion Leave</t>
+  </si>
+  <si>
+    <t>Preparing for Nxt day Exam</t>
+  </si>
+  <si>
+    <t>Chill with friends to make my mood happy and refresh</t>
+  </si>
+  <si>
+    <t>Played after so many years Cricket which make me so happy</t>
   </si>
 </sst>
 </file>
@@ -4203,115 +4221,235 @@
         <v>131</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A71" s="13"/>
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
-      <c r="G71" s="14"/>
-      <c r="H71" s="14"/>
-      <c r="I71" s="15" t="str">
+    <row r="71" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A71" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B71" s="14">
+        <v>450</v>
+      </c>
+      <c r="C71" s="14">
+        <v>60</v>
+      </c>
+      <c r="D71" s="14">
+        <v>120</v>
+      </c>
+      <c r="E71" s="14">
+        <v>30</v>
+      </c>
+      <c r="F71" s="14">
+        <v>0</v>
+      </c>
+      <c r="G71" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="H71" s="14">
+        <v>120</v>
+      </c>
+      <c r="I71" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J71" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="J71" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K71" s="16"/>
-      <c r="L71" s="16"/>
-      <c r="M71" s="16"/>
-      <c r="N71" s="17"/>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A72" s="13"/>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M71" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N71" s="17" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A72" s="13">
+        <v>46311</v>
+      </c>
+      <c r="B72" s="14">
+        <v>450</v>
+      </c>
+      <c r="C72" s="14">
+        <v>30</v>
+      </c>
+      <c r="D72" s="14">
+        <v>120</v>
+      </c>
+      <c r="E72" s="14">
+        <v>30</v>
+      </c>
+      <c r="F72" s="14">
+        <v>0</v>
+      </c>
+      <c r="G72" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="H72" s="14">
+        <v>120</v>
+      </c>
+      <c r="I72" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J72" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J72" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K72" s="16"/>
-      <c r="L72" s="16"/>
-      <c r="M72" s="16"/>
-      <c r="N72" s="17"/>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A73" s="13"/>
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="14"/>
-      <c r="H73" s="14"/>
-      <c r="I73" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M72" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N72" s="17" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A73" s="13">
+        <v>46312</v>
+      </c>
+      <c r="B73" s="14">
+        <v>450</v>
+      </c>
+      <c r="C73" s="14">
+        <v>30</v>
+      </c>
+      <c r="D73" s="14">
+        <v>0</v>
+      </c>
+      <c r="E73" s="14">
+        <v>0</v>
+      </c>
+      <c r="F73" s="14">
+        <v>0</v>
+      </c>
+      <c r="G73" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="H73" s="14">
+        <v>120</v>
+      </c>
+      <c r="I73" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J73" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J73" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
-      <c r="N73" s="17"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A74" s="13"/>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="K73" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L73" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M73" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N73" s="17" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A74" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B74" s="14">
+        <v>450</v>
+      </c>
+      <c r="C74" s="14">
+        <v>30</v>
+      </c>
+      <c r="D74" s="14">
+        <v>0</v>
+      </c>
+      <c r="E74" s="14">
+        <v>0</v>
+      </c>
+      <c r="F74" s="14">
+        <v>0</v>
+      </c>
+      <c r="G74" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="H74" s="14">
+        <v>100</v>
+      </c>
+      <c r="I74" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J74" s="15" t="str">
+        <v>580</v>
+      </c>
+      <c r="J74" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K74" s="16"/>
-      <c r="L74" s="16"/>
-      <c r="M74" s="16"/>
-      <c r="N74" s="17"/>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A75" s="13"/>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
-      <c r="D75" s="14"/>
-      <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
-      <c r="I75" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="K74" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L74" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M74" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N74" s="17" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A75" s="13">
+        <v>46314</v>
+      </c>
+      <c r="B75" s="14">
+        <v>450</v>
+      </c>
+      <c r="C75" s="14">
+        <v>30</v>
+      </c>
+      <c r="D75" s="14">
+        <v>0</v>
+      </c>
+      <c r="E75" s="14">
+        <v>0</v>
+      </c>
+      <c r="F75" s="14">
+        <v>200</v>
+      </c>
+      <c r="G75" s="14">
+        <v>4</v>
+      </c>
+      <c r="H75" s="14">
+        <v>240</v>
+      </c>
+      <c r="I75" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J75" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J75" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K75" s="16"/>
-      <c r="L75" s="16"/>
-      <c r="M75" s="16"/>
-      <c r="N75" s="17"/>
+        <v>520</v>
+      </c>
+      <c r="K75" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L75" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M75" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="N75" s="17" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="13"/>

</xml_diff>

<commit_message>
Update of 20th, 21st and 22nd October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="142">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -452,6 +452,18 @@
   </si>
   <si>
     <t>Played after so many years Cricket which make me so happy</t>
+  </si>
+  <si>
+    <t>Holiday</t>
+  </si>
+  <si>
+    <t>Doing certification courses</t>
+  </si>
+  <si>
+    <t>Today my Cisco packet software Dll verification failed after so many times for these Sir give me the remind that during end tem practical bring one backup laptops from your roomates or hostel buddy otherwise you are gone</t>
+  </si>
+  <si>
+    <t>Learning basics of Python with building projects which clearing my doubts easily and also planning my big major project which is not for showcasing it is something private</t>
   </si>
 </sst>
 </file>
@@ -4452,70 +4464,142 @@
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
-      <c r="I76" s="15" t="str">
+      <c r="A76" s="13">
+        <v>46315</v>
+      </c>
+      <c r="B76" s="14">
+        <v>450</v>
+      </c>
+      <c r="C76" s="14">
+        <v>30</v>
+      </c>
+      <c r="D76" s="14">
+        <v>60</v>
+      </c>
+      <c r="E76" s="14">
+        <v>60</v>
+      </c>
+      <c r="F76" s="14">
+        <v>0</v>
+      </c>
+      <c r="G76" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="H76" s="14">
+        <v>60</v>
+      </c>
+      <c r="I76" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J76" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="J76" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K76" s="16"/>
-      <c r="L76" s="16"/>
-      <c r="M76" s="16"/>
-      <c r="N76" s="17"/>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A77" s="13"/>
-      <c r="B77" s="14"/>
-      <c r="C77" s="14"/>
-      <c r="D77" s="14"/>
-      <c r="E77" s="14"/>
-      <c r="F77" s="14"/>
-      <c r="G77" s="14"/>
-      <c r="H77" s="14"/>
-      <c r="I77" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="K76" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L76" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M76" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N76" s="17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+      <c r="A77" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B77" s="14">
+        <v>450</v>
+      </c>
+      <c r="C77" s="14">
+        <v>30</v>
+      </c>
+      <c r="D77" s="14">
+        <v>30</v>
+      </c>
+      <c r="E77" s="14">
+        <v>60</v>
+      </c>
+      <c r="F77" s="14">
+        <v>250</v>
+      </c>
+      <c r="G77" s="14">
+        <v>5</v>
+      </c>
+      <c r="H77" s="14">
+        <v>60</v>
+      </c>
+      <c r="I77" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J77" s="15" t="str">
+        <v>880</v>
+      </c>
+      <c r="J77" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K77" s="16"/>
-      <c r="L77" s="16"/>
-      <c r="M77" s="16"/>
-      <c r="N77" s="17"/>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A78" s="13"/>
-      <c r="B78" s="14"/>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
-      <c r="H78" s="14"/>
-      <c r="I78" s="15" t="str">
+        <v>560</v>
+      </c>
+      <c r="K77" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L77" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M77" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N77" s="17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A78" s="13">
+        <v>46317</v>
+      </c>
+      <c r="B78" s="14">
+        <v>450</v>
+      </c>
+      <c r="C78" s="14">
+        <v>30</v>
+      </c>
+      <c r="D78" s="14">
+        <v>30</v>
+      </c>
+      <c r="E78" s="14">
+        <v>60</v>
+      </c>
+      <c r="F78" s="14">
+        <v>300</v>
+      </c>
+      <c r="G78" s="14">
+        <v>6</v>
+      </c>
+      <c r="H78" s="14">
+        <v>0</v>
+      </c>
+      <c r="I78" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J78" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J78" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K78" s="16"/>
-      <c r="L78" s="16"/>
-      <c r="M78" s="16"/>
-      <c r="N78" s="17"/>
+        <v>570</v>
+      </c>
+      <c r="K78" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L78" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M78" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N78" s="17" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>

</xml_diff>

<commit_message>
Update 23rd, 24th and 25th of October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="145">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -464,6 +464,15 @@
   </si>
   <si>
     <t>Learning basics of Python with building projects which clearing my doubts easily and also planning my big major project which is not for showcasing it is something private</t>
+  </si>
+  <si>
+    <t>Doing regular class and doing some practice questions to create in myself problem solving abilities and logic building using C++</t>
+  </si>
+  <si>
+    <t>Completed Networking Classes where I understand how to pratically implement DNS and Server in Cisco Packet Tracer, and We got Theme based projects which I have to make using C++</t>
+  </si>
+  <si>
+    <t>Working on my Theme based Projects using C++, taking pre recorded certification courses of Java Programming and lastly some Pratice Workbook of C++ I am solving</t>
   </si>
 </sst>
 </file>
@@ -4601,71 +4610,143 @@
         <v>141</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
-      <c r="F79" s="14"/>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-      <c r="I79" s="15" t="str">
+    <row r="79" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A79" s="13">
+        <v>46318</v>
+      </c>
+      <c r="B79" s="14">
+        <v>450</v>
+      </c>
+      <c r="C79" s="14">
+        <v>30</v>
+      </c>
+      <c r="D79" s="14">
+        <v>30</v>
+      </c>
+      <c r="E79" s="14">
+        <v>180</v>
+      </c>
+      <c r="F79" s="14">
+        <v>350</v>
+      </c>
+      <c r="G79" s="14">
+        <v>7</v>
+      </c>
+      <c r="H79" s="14">
+        <v>60</v>
+      </c>
+      <c r="I79" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J79" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J79" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K79" s="16"/>
-      <c r="L79" s="16"/>
-      <c r="M79" s="16"/>
-      <c r="N79" s="17"/>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
-      <c r="B80" s="14"/>
-      <c r="C80" s="14"/>
-      <c r="D80" s="14"/>
-      <c r="E80" s="14"/>
-      <c r="F80" s="14"/>
-      <c r="G80" s="14"/>
-      <c r="H80" s="14"/>
-      <c r="I80" s="15" t="str">
+        <v>340</v>
+      </c>
+      <c r="K79" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L79" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M79" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N79" s="17" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A80" s="13">
+        <v>46319</v>
+      </c>
+      <c r="B80" s="14">
+        <v>450</v>
+      </c>
+      <c r="C80" s="14">
+        <v>30</v>
+      </c>
+      <c r="D80" s="14">
+        <v>30</v>
+      </c>
+      <c r="E80" s="14">
+        <v>180</v>
+      </c>
+      <c r="F80" s="14">
+        <v>50</v>
+      </c>
+      <c r="G80" s="14">
+        <v>1</v>
+      </c>
+      <c r="H80" s="14">
+        <v>60</v>
+      </c>
+      <c r="I80" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J80" s="15" t="str">
+        <v>800</v>
+      </c>
+      <c r="J80" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K80" s="16"/>
-      <c r="L80" s="16"/>
-      <c r="M80" s="16"/>
-      <c r="N80" s="17"/>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A81" s="13"/>
-      <c r="B81" s="14"/>
-      <c r="C81" s="14"/>
-      <c r="D81" s="14"/>
-      <c r="E81" s="14"/>
-      <c r="F81" s="14"/>
-      <c r="G81" s="14"/>
-      <c r="H81" s="14"/>
-      <c r="I81" s="15" t="str">
+        <v>640</v>
+      </c>
+      <c r="K80" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L80" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M80" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N80" s="17" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="A81" s="13">
+        <v>46320</v>
+      </c>
+      <c r="B81" s="14">
+        <v>450</v>
+      </c>
+      <c r="C81" s="14">
+        <v>30</v>
+      </c>
+      <c r="D81" s="14">
+        <v>30</v>
+      </c>
+      <c r="E81" s="14">
+        <v>180</v>
+      </c>
+      <c r="F81" s="14">
+        <v>0</v>
+      </c>
+      <c r="G81" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="H81" s="14">
+        <v>60</v>
+      </c>
+      <c r="I81" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J81" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J81" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K81" s="16"/>
-      <c r="L81" s="16"/>
-      <c r="M81" s="16"/>
-      <c r="N81" s="17"/>
+        <v>690</v>
+      </c>
+      <c r="K81" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L81" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M81" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N81" s="17" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="13"/>

</xml_diff>

<commit_message>
Update 26th, 27th, 28th, 29th, 30th October 2026
</commit_message>
<xml_diff>
--- a/Introudction in Pyhton EXCEL/12605178.xlsx
+++ b/Introudction in Pyhton EXCEL/12605178.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="148">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -473,6 +473,15 @@
   </si>
   <si>
     <t>Working on my Theme based Projects using C++, taking pre recorded certification courses of Java Programming and lastly some Pratice Workbook of C++ I am solving</t>
+  </si>
+  <si>
+    <t>Maharishi Valmiki Holiday</t>
+  </si>
+  <si>
+    <t>Completing my certifcation s course</t>
+  </si>
+  <si>
+    <t>Preapring for CA - 2 (Data Communication and Networking)</t>
   </si>
 </sst>
 </file>
@@ -4748,115 +4757,235 @@
         <v>144</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A82" s="13"/>
-      <c r="B82" s="14"/>
-      <c r="C82" s="14"/>
-      <c r="D82" s="14"/>
-      <c r="E82" s="14"/>
-      <c r="F82" s="14"/>
-      <c r="G82" s="14"/>
-      <c r="H82" s="14"/>
-      <c r="I82" s="15" t="str">
+    <row r="82" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A82" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B82" s="14">
+        <v>450</v>
+      </c>
+      <c r="C82" s="14">
+        <v>30</v>
+      </c>
+      <c r="D82" s="14">
+        <v>30</v>
+      </c>
+      <c r="E82" s="14">
+        <v>30</v>
+      </c>
+      <c r="F82" s="14">
+        <v>0</v>
+      </c>
+      <c r="G82" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="H82" s="14">
+        <v>60</v>
+      </c>
+      <c r="I82" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J82" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J82" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K82" s="16"/>
-      <c r="L82" s="16"/>
-      <c r="M82" s="16"/>
-      <c r="N82" s="17"/>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A83" s="13"/>
-      <c r="B83" s="14"/>
-      <c r="C83" s="14"/>
-      <c r="D83" s="14"/>
-      <c r="E83" s="14"/>
-      <c r="F83" s="14"/>
-      <c r="G83" s="14"/>
-      <c r="H83" s="14"/>
-      <c r="I83" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="K82" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L82" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M82" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N82" s="17" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="A83" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B83" s="14">
+        <v>450</v>
+      </c>
+      <c r="C83" s="14">
+        <v>30</v>
+      </c>
+      <c r="D83" s="14">
+        <v>30</v>
+      </c>
+      <c r="E83" s="14">
+        <v>180</v>
+      </c>
+      <c r="F83" s="14">
+        <v>250</v>
+      </c>
+      <c r="G83" s="14">
+        <v>5</v>
+      </c>
+      <c r="H83" s="14">
+        <v>60</v>
+      </c>
+      <c r="I83" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J83" s="15" t="str">
+        <v>1000</v>
+      </c>
+      <c r="J83" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K83" s="16"/>
-      <c r="L83" s="16"/>
-      <c r="M83" s="16"/>
-      <c r="N83" s="17"/>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A84" s="13"/>
-      <c r="B84" s="14"/>
-      <c r="C84" s="14"/>
-      <c r="D84" s="14"/>
-      <c r="E84" s="14"/>
-      <c r="F84" s="14"/>
-      <c r="G84" s="14"/>
-      <c r="H84" s="14"/>
-      <c r="I84" s="15" t="str">
+        <v>440</v>
+      </c>
+      <c r="K83" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L83" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M83" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N83" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" ht="97.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="13">
+        <v>46323</v>
+      </c>
+      <c r="B84" s="14">
+        <v>450</v>
+      </c>
+      <c r="C84" s="14">
+        <v>30</v>
+      </c>
+      <c r="D84" s="14">
+        <v>30</v>
+      </c>
+      <c r="E84" s="14">
+        <v>100</v>
+      </c>
+      <c r="F84" s="14">
+        <v>250</v>
+      </c>
+      <c r="G84" s="14">
+        <v>5</v>
+      </c>
+      <c r="H84" s="14">
+        <v>60</v>
+      </c>
+      <c r="I84" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J84" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J84" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K84" s="16"/>
-      <c r="L84" s="16"/>
-      <c r="M84" s="16"/>
-      <c r="N84" s="17"/>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A85" s="13"/>
-      <c r="B85" s="14"/>
-      <c r="C85" s="14"/>
-      <c r="D85" s="14"/>
-      <c r="E85" s="14"/>
-      <c r="F85" s="14"/>
-      <c r="G85" s="14"/>
-      <c r="H85" s="14"/>
-      <c r="I85" s="15" t="str">
+        <v>520</v>
+      </c>
+      <c r="K84" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L84" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M84" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N84" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A85" s="13">
+        <v>46324</v>
+      </c>
+      <c r="B85" s="14">
+        <v>450</v>
+      </c>
+      <c r="C85" s="14">
+        <v>30</v>
+      </c>
+      <c r="D85" s="14">
+        <v>240</v>
+      </c>
+      <c r="E85" s="14">
+        <v>60</v>
+      </c>
+      <c r="F85" s="14">
+        <v>300</v>
+      </c>
+      <c r="G85" s="14">
+        <v>6</v>
+      </c>
+      <c r="H85" s="14">
+        <v>60</v>
+      </c>
+      <c r="I85" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J85" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J85" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K85" s="16"/>
-      <c r="L85" s="16"/>
-      <c r="M85" s="16"/>
-      <c r="N85" s="17"/>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A86" s="13"/>
-      <c r="B86" s="14"/>
-      <c r="C86" s="14"/>
-      <c r="D86" s="14"/>
-      <c r="E86" s="14"/>
-      <c r="F86" s="14"/>
-      <c r="G86" s="14"/>
-      <c r="H86" s="14"/>
-      <c r="I86" s="15" t="str">
+        <v>300</v>
+      </c>
+      <c r="K85" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L85" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M85" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N85" s="17" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="A86" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B86" s="14">
+        <v>450</v>
+      </c>
+      <c r="C86" s="14">
+        <v>30</v>
+      </c>
+      <c r="D86" s="14">
+        <v>30</v>
+      </c>
+      <c r="E86" s="14">
+        <v>180</v>
+      </c>
+      <c r="F86" s="14">
+        <v>350</v>
+      </c>
+      <c r="G86" s="14">
+        <v>7</v>
+      </c>
+      <c r="H86" s="14">
+        <v>60</v>
+      </c>
+      <c r="I86" s="15">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J86" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J86" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="K86" s="16"/>
-      <c r="L86" s="16"/>
-      <c r="M86" s="16"/>
-      <c r="N86" s="17"/>
+        <v>340</v>
+      </c>
+      <c r="K86" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L86" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M86" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N86" s="17" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="13"/>

</xml_diff>